<commit_message>
Signal book: KYN-KSRA NE loop-line / extra starters (14 signals)
Add 14 loop-line / UDL / extra platform starters to KYN-KSRA NE
(DN NE 63->70, UP NE 67->74) from data/KJT-KHPI/Loop-Str/LOOP STR.xlsx
via the runbook re-import path. Each loop/extra starter is placed
immediately after its platform-starter anchor and parallel-grouped
with it (parallel_group_id 1-12). VSD S-4 (long-deferred) included.
TLA S-6 added as a 2nd PF starter per user confirmation.

Also document the branch policy: all signal-book work commits to the
signal-book branch only, never master.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/KYN_KSRA/dnne_signals.xlsx
+++ b/data/KYN_KSRA/dnne_signals.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB64"/>
+  <dimension ref="A1:AB71"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -564,6 +564,12 @@
       <c r="Z2">
         <v>1</v>
       </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -632,6 +638,12 @@
       <c r="V3">
         <v>0</v>
       </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
       <c r="Y3">
         <v>300</v>
       </c>
@@ -640,12 +652,21 @@
       </c>
       <c r="AA3" t="str">
         <v>54/08</v>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>NE-5501</v>
       </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
       <c r="D4" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -703,6 +724,12 @@
       <c r="V4">
         <v>0</v>
       </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
       <c r="Y4">
         <v>300</v>
       </c>
@@ -711,12 +738,21 @@
       </c>
       <c r="AA4" t="str">
         <v>55/02</v>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>NE-5515</v>
       </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
       <c r="D5" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -774,6 +810,12 @@
       <c r="V5">
         <v>0</v>
       </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
       <c r="Y5">
         <v>300</v>
       </c>
@@ -782,12 +824,21 @@
       </c>
       <c r="AA5" t="str">
         <v>55/42</v>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
         <v>NE-5611</v>
       </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
       <c r="D6" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -845,6 +896,12 @@
       <c r="V6">
         <v>0</v>
       </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
       <c r="Y6">
         <v>300</v>
       </c>
@@ -853,12 +910,21 @@
       </c>
       <c r="AA6" t="str">
         <v>56/22</v>
+      </c>
+      <c r="AB6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>NE-5703</v>
       </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
       <c r="D7" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -916,6 +982,12 @@
       <c r="V7">
         <v>0</v>
       </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
       <c r="Y7">
         <v>300</v>
       </c>
@@ -924,12 +996,21 @@
       </c>
       <c r="AA7" t="str">
         <v>57/06</v>
+      </c>
+      <c r="AB7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
         <v>NE-5783</v>
       </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
       <c r="D8" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -987,6 +1068,12 @@
       <c r="V8">
         <v>0</v>
       </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
       <c r="Y8">
         <v>300</v>
       </c>
@@ -995,12 +1082,21 @@
       </c>
       <c r="AA8" t="str">
         <v>57/32</v>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
         <v>NE-5829</v>
       </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
       <c r="D9" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -1058,6 +1154,12 @@
       <c r="V9">
         <v>0</v>
       </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
       <c r="Y9">
         <v>300</v>
       </c>
@@ -1066,12 +1168,21 @@
       </c>
       <c r="AA9" t="str">
         <v>58/10</v>
+      </c>
+      <c r="AB9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
         <v>NE-5891</v>
       </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
       <c r="D10" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -1129,6 +1240,12 @@
       <c r="V10">
         <v>0</v>
       </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
       <c r="Y10">
         <v>300</v>
       </c>
@@ -1137,12 +1254,21 @@
       </c>
       <c r="AA10" t="str">
         <v>58/40</v>
+      </c>
+      <c r="AB10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
         <v>Gate-48</v>
       </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
       <c r="D11" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -1200,6 +1326,12 @@
       <c r="V11">
         <v>0</v>
       </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
       <c r="Y11">
         <v>250</v>
       </c>
@@ -1208,12 +1340,21 @@
       </c>
       <c r="AA11" t="str">
         <v>59/26</v>
+      </c>
+      <c r="AB11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
         <v>NE-6003</v>
       </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
       <c r="D12" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -1271,6 +1412,12 @@
       <c r="V12">
         <v>0</v>
       </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
       <c r="Y12">
         <v>330</v>
       </c>
@@ -1279,12 +1426,21 @@
       </c>
       <c r="AA12" t="str">
         <v>60/08</v>
+      </c>
+      <c r="AB12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
         <v>NE-6101</v>
       </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
       <c r="D13" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -1342,6 +1498,12 @@
       <c r="V13">
         <v>0</v>
       </c>
+      <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
       <c r="Y13">
         <v>270</v>
       </c>
@@ -1350,12 +1512,21 @@
       </c>
       <c r="AA13" t="str">
         <v>60/38</v>
+      </c>
+      <c r="AB13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
         <v>NE-6111</v>
       </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
       <c r="D14" t="str">
         <v>KYN-KSRA</v>
       </c>
@@ -1413,6 +1584,12 @@
       <c r="V14">
         <v>0</v>
       </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
       <c r="Y14">
         <v>280</v>
       </c>
@@ -1421,6 +1598,9 @@
       </c>
       <c r="AA14" t="str">
         <v>61/28</v>
+      </c>
+      <c r="AB14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1505,6 +1685,9 @@
       <c r="AA15" t="str">
         <v>62/18</v>
       </c>
+      <c r="AB15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1588,6 +1771,9 @@
       <c r="AA16" t="str">
         <v>63/42</v>
       </c>
+      <c r="AB16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1656,6 +1842,12 @@
       <c r="V17">
         <v>0</v>
       </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
       <c r="Y17">
         <v>210</v>
       </c>
@@ -1665,10 +1857,13 @@
       <c r="AA17" t="str">
         <v>PF-1 STR</v>
       </c>
+      <c r="AB17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>TLA S-8</v>
+        <v>TLA S-6</v>
       </c>
       <c r="B18" t="str">
         <v>TLA</v>
@@ -1686,16 +1881,16 @@
         <v>DN</v>
       </c>
       <c r="G18" t="str">
-        <v>64/34</v>
+        <v>PF-2 STR</v>
       </c>
       <c r="H18">
-        <v>64.494</v>
-      </c>
-      <c r="I18">
-        <v>19.30041</v>
-      </c>
-      <c r="J18">
-        <v>73.20531</v>
+        <v>64.11</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
       </c>
       <c r="K18" t="str">
         <v>Semi-Automatic</v>
@@ -1704,7 +1899,7 @@
         <v>Left</v>
       </c>
       <c r="M18" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -1733,19 +1928,34 @@
       <c r="V18">
         <v>0</v>
       </c>
-      <c r="Y18">
-        <v>250</v>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
+        <v/>
       </c>
       <c r="Z18">
         <v>1</v>
       </c>
       <c r="AA18" t="str">
-        <v>64/34</v>
+        <v>64/12</v>
+      </c>
+      <c r="AB18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Gate-52 DIST</v>
+        <v>TLA S-8</v>
+      </c>
+      <c r="B19" t="str">
+        <v>TLA</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Titwala</v>
       </c>
       <c r="D19" t="str">
         <v>KYN-KSRA</v>
@@ -1757,19 +1967,19 @@
         <v>DN</v>
       </c>
       <c r="G19" t="str">
-        <v>65/04</v>
+        <v>64/34</v>
       </c>
       <c r="H19">
-        <v>65.045</v>
+        <v>64.494</v>
       </c>
       <c r="I19">
-        <v>19.30306</v>
+        <v>19.30041</v>
       </c>
       <c r="J19">
-        <v>73.20973</v>
+        <v>73.20531</v>
       </c>
       <c r="K19" t="str">
-        <v>Manual</v>
+        <v>Semi-Automatic</v>
       </c>
       <c r="L19" t="str">
         <v>Left</v>
@@ -1804,22 +2014,34 @@
       <c r="V19">
         <v>0</v>
       </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
       <c r="Y19">
-        <v>540</v>
+        <v>250</v>
       </c>
       <c r="Z19">
         <v>1</v>
       </c>
       <c r="AA19" t="str">
-        <v>65/04</v>
+        <v>64/34</v>
       </c>
       <c r="AB19" t="str">
-        <v>Distant</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Gate-52</v>
+        <v>Gate-52 DIST</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
       </c>
       <c r="D20" t="str">
         <v>KYN-KSRA</v>
@@ -1831,25 +2053,25 @@
         <v>DN</v>
       </c>
       <c r="G20" t="str">
-        <v>66/08</v>
+        <v>65/04</v>
       </c>
       <c r="H20">
-        <v>66.055</v>
+        <v>65.045</v>
       </c>
       <c r="I20">
-        <v>19.31004</v>
+        <v>19.30306</v>
       </c>
       <c r="J20">
-        <v>73.21548</v>
+        <v>73.20973</v>
       </c>
       <c r="K20" t="str">
-        <v>Gate</v>
+        <v>Manual</v>
       </c>
       <c r="L20" t="str">
         <v>Left</v>
       </c>
       <c r="M20" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -1878,19 +2100,34 @@
       <c r="V20">
         <v>0</v>
       </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+      <c r="X20" t="str">
+        <v/>
+      </c>
       <c r="Y20">
-        <v>320</v>
+        <v>540</v>
       </c>
       <c r="Z20">
         <v>1</v>
       </c>
       <c r="AA20" t="str">
-        <v>66/08</v>
+        <v>65/04</v>
+      </c>
+      <c r="AB20" t="str">
+        <v>Distant</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>TLA IBS DIST</v>
+        <v>Gate-52</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
       </c>
       <c r="D21" t="str">
         <v>KYN-KSRA</v>
@@ -1902,19 +2139,19 @@
         <v>DN</v>
       </c>
       <c r="G21" t="str">
-        <v>66/46</v>
+        <v>66/08</v>
       </c>
       <c r="H21">
-        <v>66.739</v>
+        <v>66.055</v>
       </c>
       <c r="I21">
-        <v>19.31605</v>
+        <v>19.31004</v>
       </c>
       <c r="J21">
-        <v>73.21633</v>
+        <v>73.21548</v>
       </c>
       <c r="K21" t="str">
-        <v>Manual</v>
+        <v>Gate</v>
       </c>
       <c r="L21" t="str">
         <v>Left</v>
@@ -1949,22 +2186,34 @@
       <c r="V21">
         <v>0</v>
       </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+      <c r="X21" t="str">
+        <v/>
+      </c>
       <c r="Y21">
-        <v>450</v>
+        <v>320</v>
       </c>
       <c r="Z21">
         <v>1</v>
       </c>
       <c r="AA21" t="str">
-        <v>66/46</v>
+        <v>66/08</v>
       </c>
       <c r="AB21" t="str">
-        <v>Distant</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>TLA S-9</v>
+        <v>TLA IBS DIST</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v/>
       </c>
       <c r="D22" t="str">
         <v>KYN-KSRA</v>
@@ -1976,16 +2225,16 @@
         <v>DN</v>
       </c>
       <c r="G22" t="str">
-        <v>67/50</v>
+        <v>66/46</v>
       </c>
       <c r="H22">
-        <v>67.889</v>
+        <v>66.739</v>
       </c>
       <c r="I22">
-        <v>19.32631</v>
+        <v>19.31605</v>
       </c>
       <c r="J22">
-        <v>73.21514</v>
+        <v>73.21633</v>
       </c>
       <c r="K22" t="str">
         <v>Manual</v>
@@ -1994,7 +2243,7 @@
         <v>Left</v>
       </c>
       <c r="M22" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -2022,6 +2271,12 @@
       </c>
       <c r="V22">
         <v>0</v>
+      </c>
+      <c r="W22" t="str">
+        <v/>
+      </c>
+      <c r="X22" t="str">
+        <v/>
       </c>
       <c r="Y22">
         <v>450</v>
@@ -2030,15 +2285,21 @@
         <v>1</v>
       </c>
       <c r="AA22" t="str">
-        <v>67/50</v>
+        <v>66/46</v>
       </c>
       <c r="AB22" t="str">
-        <v>IBS</v>
+        <v>Distant</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Gate-55</v>
+        <v>TLA S-9</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v/>
       </c>
       <c r="D23" t="str">
         <v>KYN-KSRA</v>
@@ -2050,19 +2311,19 @@
         <v>DN</v>
       </c>
       <c r="G23" t="str">
-        <v>69/18</v>
+        <v>67/50</v>
       </c>
       <c r="H23">
-        <v>69.439</v>
+        <v>67.889</v>
       </c>
       <c r="I23">
-        <v>19.34005</v>
+        <v>19.32631</v>
       </c>
       <c r="J23">
-        <v>73.21352</v>
+        <v>73.21514</v>
       </c>
       <c r="K23" t="str">
-        <v>Gate</v>
+        <v>Manual</v>
       </c>
       <c r="L23" t="str">
         <v>Left</v>
@@ -2097,25 +2358,34 @@
       <c r="V23">
         <v>0</v>
       </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
       <c r="Y23">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="Z23">
         <v>1</v>
       </c>
       <c r="AA23" t="str">
-        <v>69/18</v>
+        <v>67/50</v>
+      </c>
+      <c r="AB23" t="str">
+        <v>IBS</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>KDV S-3</v>
+        <v>Gate-55</v>
       </c>
       <c r="B24" t="str">
-        <v>KDV</v>
+        <v/>
       </c>
       <c r="C24" t="str">
-        <v>Khadavli</v>
+        <v/>
       </c>
       <c r="D24" t="str">
         <v>KYN-KSRA</v>
@@ -2127,25 +2397,25 @@
         <v>DN</v>
       </c>
       <c r="G24" t="str">
-        <v>70/42</v>
+        <v>69/18</v>
       </c>
       <c r="H24">
-        <v>70.799</v>
+        <v>69.439</v>
       </c>
       <c r="I24">
-        <v>19.35209</v>
+        <v>19.34005</v>
       </c>
       <c r="J24">
-        <v>73.21301</v>
+        <v>73.21352</v>
       </c>
       <c r="K24" t="str">
-        <v>Manual</v>
+        <v>Gate</v>
       </c>
       <c r="L24" t="str">
         <v>Left</v>
       </c>
       <c r="M24" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -2163,39 +2433,39 @@
         <v>0</v>
       </c>
       <c r="S24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T24">
         <v>0</v>
       </c>
       <c r="U24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V24">
         <v>0</v>
       </c>
       <c r="W24" t="str">
-        <v>RI:L1= DN LL</v>
+        <v/>
       </c>
       <c r="X24" t="str">
-        <v>Book shows one left arm on top of vertical stem</v>
+        <v/>
       </c>
       <c r="Y24">
-        <v>350</v>
+        <v>600</v>
       </c>
       <c r="Z24">
         <v>1</v>
       </c>
       <c r="AA24" t="str">
-        <v>70/42</v>
+        <v>69/18</v>
       </c>
       <c r="AB24" t="str">
-        <v>Home</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>KDV S-12</v>
+        <v>KDV S-3</v>
       </c>
       <c r="B25" t="str">
         <v>KDV</v>
@@ -2213,25 +2483,25 @@
         <v>DN</v>
       </c>
       <c r="G25" t="str">
-        <v>72/10</v>
+        <v>70/42</v>
       </c>
       <c r="H25">
-        <v>72.129</v>
+        <v>70.799</v>
       </c>
       <c r="I25">
-        <v>19.35858</v>
+        <v>19.35209</v>
       </c>
       <c r="J25">
-        <v>73.22317</v>
+        <v>73.21301</v>
       </c>
       <c r="K25" t="str">
         <v>Manual</v>
       </c>
       <c r="L25" t="str">
-        <v>Gantry</v>
+        <v>Left</v>
       </c>
       <c r="M25" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="N25">
         <v>0</v>
@@ -2249,33 +2519,39 @@
         <v>0</v>
       </c>
       <c r="S25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T25">
         <v>0</v>
       </c>
       <c r="U25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V25">
         <v>0</v>
       </c>
+      <c r="W25" t="str">
+        <v>RI:L1= DN LL</v>
+      </c>
+      <c r="X25" t="str">
+        <v>Book shows one left arm on top of vertical stem</v>
+      </c>
       <c r="Y25">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="Z25">
         <v>1</v>
       </c>
       <c r="AA25" t="str">
-        <v>72/10</v>
+        <v>70/42</v>
       </c>
       <c r="AB25" t="str">
-        <v>Starter</v>
+        <v>Home</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>KDV S-13</v>
+        <v>KDV S-12</v>
       </c>
       <c r="B26" t="str">
         <v>KDV</v>
@@ -2293,25 +2569,25 @@
         <v>DN</v>
       </c>
       <c r="G26" t="str">
-        <v>72/36</v>
+        <v>72/10</v>
       </c>
       <c r="H26">
-        <v>72.589</v>
+        <v>72.129</v>
       </c>
       <c r="I26">
-        <v>19.36122</v>
+        <v>19.35858</v>
       </c>
       <c r="J26">
-        <v>73.22654</v>
+        <v>73.22317</v>
       </c>
       <c r="K26" t="str">
         <v>Manual</v>
       </c>
       <c r="L26" t="str">
-        <v>Left</v>
+        <v>Gantry</v>
       </c>
       <c r="M26" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="N26">
         <v>0</v>
@@ -2339,6 +2615,12 @@
       </c>
       <c r="V26">
         <v>0</v>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+      <c r="X26" t="str">
+        <v/>
       </c>
       <c r="Y26">
         <v>300</v>
@@ -2347,15 +2629,21 @@
         <v>1</v>
       </c>
       <c r="AA26" t="str">
-        <v>72/36</v>
+        <v>72/10</v>
       </c>
       <c r="AB26" t="str">
-        <v>Advance Starter</v>
+        <v>Starter</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>KDV IBS DIST</v>
+        <v>KDV S-11</v>
+      </c>
+      <c r="B27" t="str">
+        <v>KDV</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Khadavli</v>
       </c>
       <c r="D27" t="str">
         <v>KYN-KSRA</v>
@@ -2367,16 +2655,16 @@
         <v>DN</v>
       </c>
       <c r="G27" t="str">
-        <v>74/18</v>
-      </c>
-      <c r="H27">
-        <v>74.459</v>
-      </c>
-      <c r="I27">
-        <v>19.37323</v>
-      </c>
-      <c r="J27">
-        <v>73.23897</v>
+        <v>DN LOOP STR</v>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
       </c>
       <c r="K27" t="str">
         <v>Manual</v>
@@ -2385,7 +2673,7 @@
         <v>Left</v>
       </c>
       <c r="M27" t="str">
-        <v>Unknown</v>
+        <v/>
       </c>
       <c r="N27">
         <v>0</v>
@@ -2414,22 +2702,34 @@
       <c r="V27">
         <v>0</v>
       </c>
-      <c r="Y27">
-        <v>480</v>
+      <c r="W27" t="str">
+        <v/>
+      </c>
+      <c r="X27" t="str">
+        <v/>
+      </c>
+      <c r="Y27" t="str">
+        <v/>
       </c>
       <c r="Z27">
         <v>1</v>
       </c>
       <c r="AA27" t="str">
-        <v>74/18</v>
+        <v>72/10</v>
       </c>
       <c r="AB27" t="str">
-        <v>IBS Distant</v>
+        <v>Starter (Loop)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>KDV S-14</v>
+        <v>KDV S-13</v>
+      </c>
+      <c r="B28" t="str">
+        <v>KDV</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Khadavli</v>
       </c>
       <c r="D28" t="str">
         <v>KYN-KSRA</v>
@@ -2441,16 +2741,16 @@
         <v>DN</v>
       </c>
       <c r="G28" t="str">
-        <v>75/18</v>
+        <v>72/36</v>
       </c>
       <c r="H28">
-        <v>75.499</v>
+        <v>72.589</v>
       </c>
       <c r="I28">
-        <v>19.38041</v>
+        <v>19.36122</v>
       </c>
       <c r="J28">
-        <v>73.24516</v>
+        <v>73.22654</v>
       </c>
       <c r="K28" t="str">
         <v>Manual</v>
@@ -2459,7 +2759,7 @@
         <v>Left</v>
       </c>
       <c r="M28" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="N28">
         <v>0</v>
@@ -2488,28 +2788,34 @@
       <c r="V28">
         <v>0</v>
       </c>
+      <c r="W28" t="str">
+        <v/>
+      </c>
+      <c r="X28" t="str">
+        <v/>
+      </c>
       <c r="Y28">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="Z28">
         <v>1</v>
       </c>
       <c r="AA28" t="str">
-        <v>75/18</v>
+        <v>72/36</v>
       </c>
       <c r="AB28" t="str">
-        <v>IBS</v>
+        <v>Advance Starter</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>VSD DIST</v>
+        <v>KDV IBS DIST</v>
       </c>
       <c r="B29" t="str">
-        <v>VSD</v>
+        <v/>
       </c>
       <c r="C29" t="str">
-        <v>Vasind</v>
+        <v/>
       </c>
       <c r="D29" t="str">
         <v>KYN-KSRA</v>
@@ -2521,16 +2827,16 @@
         <v>DN</v>
       </c>
       <c r="G29" t="str">
-        <v>77/6</v>
+        <v>74/18</v>
       </c>
       <c r="H29">
-        <v>76.899</v>
+        <v>74.459</v>
       </c>
       <c r="I29">
-        <v>19.39144</v>
+        <v>19.37323</v>
       </c>
       <c r="J29">
-        <v>73.25479</v>
+        <v>73.23897</v>
       </c>
       <c r="K29" t="str">
         <v>Manual</v>
@@ -2539,7 +2845,7 @@
         <v>Left</v>
       </c>
       <c r="M29" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="N29">
         <v>0</v>
@@ -2568,28 +2874,34 @@
       <c r="V29">
         <v>0</v>
       </c>
+      <c r="W29" t="str">
+        <v/>
+      </c>
+      <c r="X29" t="str">
+        <v/>
+      </c>
       <c r="Y29">
-        <v>500</v>
+        <v>480</v>
       </c>
       <c r="Z29">
         <v>1</v>
       </c>
       <c r="AA29" t="str">
-        <v>77/6</v>
+        <v>74/18</v>
       </c>
       <c r="AB29" t="str">
-        <v>Distant</v>
+        <v>IBS Distant</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>VSD S-2</v>
+        <v>KDV S-14</v>
       </c>
       <c r="B30" t="str">
-        <v>VSD</v>
+        <v/>
       </c>
       <c r="C30" t="str">
-        <v>Vasind</v>
+        <v/>
       </c>
       <c r="D30" t="str">
         <v>KYN-KSRA</v>
@@ -2601,16 +2913,16 @@
         <v>DN</v>
       </c>
       <c r="G30" t="str">
-        <v>78/22</v>
+        <v>75/18</v>
       </c>
       <c r="H30">
-        <v>78.249</v>
+        <v>75.499</v>
       </c>
       <c r="I30">
-        <v>19.40037</v>
+        <v>19.38041</v>
       </c>
       <c r="J30">
-        <v>73.25928</v>
+        <v>73.24516</v>
       </c>
       <c r="K30" t="str">
         <v>Manual</v>
@@ -2637,39 +2949,39 @@
         <v>0</v>
       </c>
       <c r="S30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T30">
         <v>0</v>
       </c>
       <c r="U30">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V30">
         <v>0</v>
       </c>
       <c r="W30" t="str">
-        <v>RI:L1= DN LL; L2=UDL</v>
+        <v/>
       </c>
       <c r="X30" t="str">
-        <v>Book shows two left arms on top of vertical stem</v>
+        <v/>
       </c>
       <c r="Y30">
-        <v>310</v>
+        <v>350</v>
       </c>
       <c r="Z30">
         <v>1</v>
       </c>
       <c r="AA30" t="str">
-        <v>78/22</v>
+        <v>75/18</v>
       </c>
       <c r="AB30" t="str">
-        <v>Home</v>
+        <v>IBS</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>VSD S-3</v>
+        <v>VSD DIST</v>
       </c>
       <c r="B31" t="str">
         <v>VSD</v>
@@ -2687,25 +2999,25 @@
         <v>DN</v>
       </c>
       <c r="G31" t="str">
-        <v>79/34</v>
+        <v>77/6</v>
       </c>
       <c r="H31">
-        <v>79.459</v>
+        <v>76.899</v>
       </c>
       <c r="I31">
-        <v>19.40851</v>
+        <v>19.39144</v>
       </c>
       <c r="J31">
-        <v>73.26995</v>
+        <v>73.25479</v>
       </c>
       <c r="K31" t="str">
         <v>Manual</v>
       </c>
       <c r="L31" t="str">
-        <v>Extreme Left</v>
+        <v>Left</v>
       </c>
       <c r="M31" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -2714,10 +3026,10 @@
         <v>0</v>
       </c>
       <c r="P31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R31">
         <v>0</v>
@@ -2734,22 +3046,28 @@
       <c r="V31">
         <v>0</v>
       </c>
+      <c r="W31" t="str">
+        <v/>
+      </c>
+      <c r="X31" t="str">
+        <v/>
+      </c>
       <c r="Y31">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="Z31">
         <v>1</v>
       </c>
       <c r="AA31" t="str">
-        <v>79/34</v>
+        <v>77/6</v>
       </c>
       <c r="AB31" t="str">
-        <v>Starter</v>
+        <v>Distant</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>VSD S-11</v>
+        <v>VSD S-2</v>
       </c>
       <c r="B32" t="str">
         <v>VSD</v>
@@ -2767,16 +3085,16 @@
         <v>DN</v>
       </c>
       <c r="G32" t="str">
-        <v>80/02</v>
+        <v>78/22</v>
       </c>
       <c r="H32">
-        <v>79.856</v>
+        <v>78.249</v>
       </c>
       <c r="I32">
-        <v>19.40936</v>
+        <v>19.40037</v>
       </c>
       <c r="J32">
-        <v>73.27362</v>
+        <v>73.25928</v>
       </c>
       <c r="K32" t="str">
         <v>Manual</v>
@@ -2803,33 +3121,45 @@
         <v>0</v>
       </c>
       <c r="S32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T32">
         <v>0</v>
       </c>
       <c r="U32">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V32">
         <v>0</v>
       </c>
+      <c r="W32" t="str">
+        <v>RI:L1= DN LL; L2=UDL</v>
+      </c>
+      <c r="X32" t="str">
+        <v>Book shows two left arms on top of vertical stem</v>
+      </c>
       <c r="Y32">
-        <v>350</v>
+        <v>310</v>
       </c>
       <c r="Z32">
         <v>1</v>
       </c>
       <c r="AA32" t="str">
-        <v>80/02</v>
+        <v>78/22</v>
       </c>
       <c r="AB32" t="str">
-        <v>Advance Starter</v>
+        <v>Home</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Gate-64</v>
+        <v>VSD S-3</v>
+      </c>
+      <c r="B33" t="str">
+        <v>VSD</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Vasind</v>
       </c>
       <c r="D33" t="str">
         <v>KYN-KSRA</v>
@@ -2841,22 +3171,22 @@
         <v>DN</v>
       </c>
       <c r="G33" t="str">
-        <v>80/22</v>
+        <v>79/34</v>
       </c>
       <c r="H33">
-        <v>80.309</v>
+        <v>79.459</v>
       </c>
       <c r="I33">
-        <v>19.4102</v>
+        <v>19.40851</v>
       </c>
       <c r="J33">
-        <v>73.27783</v>
+        <v>73.26995</v>
       </c>
       <c r="K33" t="str">
-        <v>Gate</v>
+        <v>Manual</v>
       </c>
       <c r="L33" t="str">
-        <v>Left</v>
+        <v>Extreme Left</v>
       </c>
       <c r="M33" t="str">
         <v>Unknown</v>
@@ -2868,10 +3198,10 @@
         <v>0</v>
       </c>
       <c r="P33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R33">
         <v>0</v>
@@ -2888,19 +3218,34 @@
       <c r="V33">
         <v>0</v>
       </c>
+      <c r="W33" t="str">
+        <v/>
+      </c>
+      <c r="X33" t="str">
+        <v/>
+      </c>
       <c r="Y33">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="Z33">
         <v>1</v>
       </c>
       <c r="AA33" t="str">
-        <v>80/22</v>
+        <v>79/34</v>
+      </c>
+      <c r="AB33" t="str">
+        <v>Starter</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>VSD S-12</v>
+        <v>VSD S-4</v>
+      </c>
+      <c r="B34" t="str">
+        <v>VSD</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Vasind</v>
       </c>
       <c r="D34" t="str">
         <v>KYN-KSRA</v>
@@ -2912,16 +3257,16 @@
         <v>DN</v>
       </c>
       <c r="G34" t="str">
-        <v>81/46</v>
-      </c>
-      <c r="H34">
-        <v>81.819</v>
-      </c>
-      <c r="I34">
-        <v>19.41549</v>
-      </c>
-      <c r="J34">
-        <v>73.29093</v>
+        <v>DN LOOP STR</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
       </c>
       <c r="K34" t="str">
         <v>Manual</v>
@@ -2930,7 +3275,7 @@
         <v>Left</v>
       </c>
       <c r="M34" t="str">
-        <v>Unknown</v>
+        <v/>
       </c>
       <c r="N34">
         <v>0</v>
@@ -2951,7 +3296,7 @@
         <v>0</v>
       </c>
       <c r="T34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U34">
         <v>0</v>
@@ -2959,28 +3304,34 @@
       <c r="V34">
         <v>0</v>
       </c>
-      <c r="Y34">
-        <v>600</v>
+      <c r="W34" t="str">
+        <v/>
+      </c>
+      <c r="X34" t="str">
+        <v/>
+      </c>
+      <c r="Y34" t="str">
+        <v/>
       </c>
       <c r="Z34">
         <v>1</v>
       </c>
       <c r="AA34" t="str">
-        <v>81/46</v>
+        <v>VSD 1040</v>
       </c>
       <c r="AB34" t="str">
-        <v>IBS</v>
+        <v>Starter (Loop)</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ASO DIST</v>
+        <v>VSD S-5</v>
       </c>
       <c r="B35" t="str">
-        <v>ASO</v>
+        <v>VSD</v>
       </c>
       <c r="C35" t="str">
-        <v>Asangaon</v>
+        <v>Vasind</v>
       </c>
       <c r="D35" t="str">
         <v>KYN-KSRA</v>
@@ -2992,16 +3343,16 @@
         <v>DN</v>
       </c>
       <c r="G35" t="str">
-        <v>83/24</v>
-      </c>
-      <c r="H35">
-        <v>83.279</v>
-      </c>
-      <c r="I35">
-        <v>19.4254</v>
-      </c>
-      <c r="J35">
-        <v>73.29932</v>
+        <v>UDL DN STR</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
       </c>
       <c r="K35" t="str">
         <v>Manual</v>
@@ -3010,7 +3361,7 @@
         <v>Left</v>
       </c>
       <c r="M35" t="str">
-        <v>Unknown</v>
+        <v/>
       </c>
       <c r="N35">
         <v>0</v>
@@ -3039,28 +3390,34 @@
       <c r="V35">
         <v>0</v>
       </c>
-      <c r="Y35">
-        <v>600</v>
+      <c r="W35" t="str">
+        <v/>
+      </c>
+      <c r="X35" t="str">
+        <v/>
+      </c>
+      <c r="Y35" t="str">
+        <v/>
       </c>
       <c r="Z35">
         <v>1</v>
       </c>
       <c r="AA35" t="str">
-        <v>83/24</v>
+        <v>VSD 1042</v>
       </c>
       <c r="AB35" t="str">
-        <v>Distant</v>
+        <v>Starter (Loop)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ASO S-2</v>
+        <v>VSD S-11</v>
       </c>
       <c r="B36" t="str">
-        <v>ASO</v>
+        <v>VSD</v>
       </c>
       <c r="C36" t="str">
-        <v>Asangaon</v>
+        <v>Vasind</v>
       </c>
       <c r="D36" t="str">
         <v>KYN-KSRA</v>
@@ -3072,34 +3429,34 @@
         <v>DN</v>
       </c>
       <c r="G36" t="str">
-        <v>84/24</v>
+        <v>80/02</v>
       </c>
       <c r="H36">
-        <v>84.299</v>
+        <v>79.856</v>
       </c>
       <c r="I36">
-        <v>19.43314</v>
+        <v>19.40936</v>
       </c>
       <c r="J36">
-        <v>73.30443</v>
+        <v>73.27362</v>
       </c>
       <c r="K36" t="str">
         <v>Manual</v>
       </c>
       <c r="L36" t="str">
-        <v>Extreme Right</v>
+        <v>Left</v>
       </c>
       <c r="M36" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="N36">
         <v>0</v>
       </c>
       <c r="O36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q36">
         <v>0</v>
@@ -3108,45 +3465,45 @@
         <v>0</v>
       </c>
       <c r="S36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T36">
         <v>0</v>
       </c>
       <c r="U36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W36" t="str">
-        <v>RI:L1= DN LL; R1=PF-2</v>
+        <v/>
       </c>
       <c r="X36" t="str">
-        <v>Book shows one left and one right arm on top of vertical stem</v>
+        <v/>
       </c>
       <c r="Y36">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="Z36">
         <v>1</v>
       </c>
       <c r="AA36" t="str">
-        <v>84/24</v>
+        <v>80/02</v>
       </c>
       <c r="AB36" t="str">
-        <v>Home</v>
+        <v>Advance Starter</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ASO S-7</v>
+        <v>Gate-64</v>
       </c>
       <c r="B37" t="str">
-        <v>ASO</v>
+        <v/>
       </c>
       <c r="C37" t="str">
-        <v>Asangaon</v>
+        <v/>
       </c>
       <c r="D37" t="str">
         <v>KYN-KSRA</v>
@@ -3158,34 +3515,34 @@
         <v>DN</v>
       </c>
       <c r="G37" t="str">
-        <v>85/34</v>
+        <v>80/22</v>
       </c>
       <c r="H37">
-        <v>85.479</v>
+        <v>80.309</v>
       </c>
       <c r="I37">
-        <v>19.44263</v>
+        <v>19.4102</v>
       </c>
       <c r="J37">
-        <v>73.30909</v>
+        <v>73.27783</v>
       </c>
       <c r="K37" t="str">
-        <v>Manual</v>
+        <v>Gate</v>
       </c>
       <c r="L37" t="str">
-        <v>Extreme Right</v>
+        <v>Left</v>
       </c>
       <c r="M37" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="N37">
         <v>0</v>
       </c>
       <c r="O37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q37">
         <v>0</v>
@@ -3205,28 +3562,34 @@
       <c r="V37">
         <v>0</v>
       </c>
+      <c r="W37" t="str">
+        <v/>
+      </c>
+      <c r="X37" t="str">
+        <v/>
+      </c>
       <c r="Y37">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="Z37">
         <v>1</v>
       </c>
       <c r="AA37" t="str">
-        <v>85/34</v>
+        <v>80/22</v>
       </c>
       <c r="AB37" t="str">
-        <v>Starter</v>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ASO S-12</v>
+        <v>VSD S-12</v>
       </c>
       <c r="B38" t="str">
-        <v>ASO</v>
+        <v/>
       </c>
       <c r="C38" t="str">
-        <v>Asangaon</v>
+        <v/>
       </c>
       <c r="D38" t="str">
         <v>KYN-KSRA</v>
@@ -3238,16 +3601,16 @@
         <v>DN</v>
       </c>
       <c r="G38" t="str">
-        <v>86/10</v>
+        <v>81/46</v>
       </c>
       <c r="H38">
-        <v>85.87299999999999</v>
+        <v>81.819</v>
       </c>
       <c r="I38">
-        <v>19.4461</v>
+        <v>19.41549</v>
       </c>
       <c r="J38">
-        <v>73.3097</v>
+        <v>73.29093</v>
       </c>
       <c r="K38" t="str">
         <v>Manual</v>
@@ -3256,7 +3619,7 @@
         <v>Left</v>
       </c>
       <c r="M38" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="N38">
         <v>0</v>
@@ -3285,22 +3648,34 @@
       <c r="V38">
         <v>0</v>
       </c>
+      <c r="W38" t="str">
+        <v/>
+      </c>
+      <c r="X38" t="str">
+        <v/>
+      </c>
       <c r="Y38">
-        <v>350</v>
+        <v>600</v>
       </c>
       <c r="Z38">
         <v>1</v>
       </c>
       <c r="AA38" t="str">
-        <v>86/10</v>
+        <v>81/46</v>
       </c>
       <c r="AB38" t="str">
-        <v>Advance Starter</v>
+        <v>IBS</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ASO IBS DIST</v>
+        <v>ASO DIST</v>
+      </c>
+      <c r="B39" t="str">
+        <v>ASO</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Asangaon</v>
       </c>
       <c r="D39" t="str">
         <v>KYN-KSRA</v>
@@ -3312,16 +3687,16 @@
         <v>DN</v>
       </c>
       <c r="G39" t="str">
-        <v>89/2</v>
+        <v>83/24</v>
       </c>
       <c r="H39">
-        <v>88.833</v>
+        <v>83.279</v>
       </c>
       <c r="I39">
-        <v>19.47014</v>
+        <v>19.4254</v>
       </c>
       <c r="J39">
-        <v>73.30104</v>
+        <v>73.29932</v>
       </c>
       <c r="K39" t="str">
         <v>Manual</v>
@@ -3330,7 +3705,7 @@
         <v>Left</v>
       </c>
       <c r="M39" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="N39">
         <v>0</v>
@@ -3358,6 +3733,12 @@
       </c>
       <c r="V39">
         <v>0</v>
+      </c>
+      <c r="W39" t="str">
+        <v/>
+      </c>
+      <c r="X39" t="str">
+        <v/>
       </c>
       <c r="Y39">
         <v>600</v>
@@ -3366,15 +3747,21 @@
         <v>1</v>
       </c>
       <c r="AA39" t="str">
-        <v>89/2</v>
+        <v>83/24</v>
       </c>
       <c r="AB39" t="str">
-        <v>IBS Distant</v>
+        <v>Distant</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ASO S-14</v>
+        <v>ASO S-2</v>
+      </c>
+      <c r="B40" t="str">
+        <v>ASO</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Asangaon</v>
       </c>
       <c r="D40" t="str">
         <v>KYN-KSRA</v>
@@ -3386,34 +3773,34 @@
         <v>DN</v>
       </c>
       <c r="G40" t="str">
-        <v>90/12</v>
+        <v>84/24</v>
       </c>
       <c r="H40">
-        <v>90.033</v>
+        <v>84.299</v>
       </c>
       <c r="I40">
-        <v>19.47645</v>
+        <v>19.43314</v>
       </c>
       <c r="J40">
-        <v>73.30968</v>
+        <v>73.30443</v>
       </c>
       <c r="K40" t="str">
         <v>Manual</v>
       </c>
       <c r="L40" t="str">
-        <v>Left</v>
+        <v>Extreme Right</v>
       </c>
       <c r="M40" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="N40">
         <v>0</v>
       </c>
       <c r="O40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q40">
         <v>0</v>
@@ -3422,33 +3809,45 @@
         <v>0</v>
       </c>
       <c r="S40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T40">
         <v>0</v>
       </c>
       <c r="U40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V40">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="W40" t="str">
+        <v>RI:L1= DN LL; R1=PF-2</v>
+      </c>
+      <c r="X40" t="str">
+        <v>Book shows one left and one right arm on top of vertical stem</v>
       </c>
       <c r="Y40">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="Z40">
         <v>1</v>
       </c>
       <c r="AA40" t="str">
-        <v>90/12</v>
+        <v>84/24</v>
       </c>
       <c r="AB40" t="str">
-        <v>IBS</v>
+        <v>Home</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Gate-69 DIST</v>
+        <v>ASO S-7</v>
+      </c>
+      <c r="B41" t="str">
+        <v>ASO</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Asangaon</v>
       </c>
       <c r="D41" t="str">
         <v>KYN-KSRA</v>
@@ -3460,34 +3859,34 @@
         <v>DN</v>
       </c>
       <c r="G41" t="str">
-        <v>91/44</v>
+        <v>85/34</v>
       </c>
       <c r="H41">
-        <v>91.613</v>
+        <v>85.479</v>
       </c>
       <c r="I41">
-        <v>19.48589</v>
+        <v>19.44263</v>
       </c>
       <c r="J41">
-        <v>73.31983</v>
+        <v>73.30909</v>
       </c>
       <c r="K41" t="str">
         <v>Manual</v>
       </c>
       <c r="L41" t="str">
-        <v>Left</v>
+        <v>Extreme Right</v>
       </c>
       <c r="M41" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="N41">
         <v>0</v>
       </c>
       <c r="O41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q41">
         <v>0</v>
@@ -3507,22 +3906,34 @@
       <c r="V41">
         <v>0</v>
       </c>
+      <c r="W41" t="str">
+        <v/>
+      </c>
+      <c r="X41" t="str">
+        <v/>
+      </c>
       <c r="Y41">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="Z41">
         <v>1</v>
       </c>
       <c r="AA41" t="str">
-        <v>91/44</v>
+        <v>85/34</v>
       </c>
       <c r="AB41" t="str">
-        <v>Distant</v>
+        <v>Starter</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Gate-69</v>
+        <v>ASO S-6</v>
+      </c>
+      <c r="B42" t="str">
+        <v>ASO</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Asangaon</v>
       </c>
       <c r="D42" t="str">
         <v>KYN-KSRA</v>
@@ -3534,34 +3945,34 @@
         <v>DN</v>
       </c>
       <c r="G42" t="str">
-        <v>92/40</v>
-      </c>
-      <c r="H42">
-        <v>92.60900000000001</v>
-      </c>
-      <c r="I42">
-        <v>19.4873</v>
-      </c>
-      <c r="J42">
-        <v>73.32914</v>
+        <v>DN LOOP STR</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
       </c>
       <c r="K42" t="str">
-        <v>Gate</v>
+        <v>Manual</v>
       </c>
       <c r="L42" t="str">
-        <v>Extreme Right</v>
+        <v>Left</v>
       </c>
       <c r="M42" t="str">
-        <v>Left</v>
+        <v/>
       </c>
       <c r="N42">
         <v>0</v>
       </c>
       <c r="O42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q42">
         <v>0</v>
@@ -3581,25 +3992,34 @@
       <c r="V42">
         <v>0</v>
       </c>
-      <c r="Y42">
-        <v>300</v>
+      <c r="W42" t="str">
+        <v/>
+      </c>
+      <c r="X42" t="str">
+        <v/>
+      </c>
+      <c r="Y42" t="str">
+        <v/>
       </c>
       <c r="Z42">
         <v>1</v>
       </c>
       <c r="AA42" t="str">
-        <v>92/40</v>
+        <v>85/40</v>
+      </c>
+      <c r="AB42" t="str">
+        <v>Starter (Loop)</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ATG S-3</v>
+        <v>ASO S-12</v>
       </c>
       <c r="B43" t="str">
-        <v>ATG</v>
+        <v>ASO</v>
       </c>
       <c r="C43" t="str">
-        <v>Atgaon</v>
+        <v>Asangaon</v>
       </c>
       <c r="D43" t="str">
         <v>KYN-KSRA</v>
@@ -3611,22 +4031,22 @@
         <v>DN</v>
       </c>
       <c r="G43" t="str">
-        <v>94/18</v>
+        <v>86/10</v>
       </c>
       <c r="H43">
-        <v>94.089</v>
+        <v>85.87299999999999</v>
       </c>
       <c r="I43">
-        <v>19.4989</v>
+        <v>19.4461</v>
       </c>
       <c r="J43">
-        <v>73.33237</v>
+        <v>73.3097</v>
       </c>
       <c r="K43" t="str">
         <v>Manual</v>
       </c>
       <c r="L43" t="str">
-        <v>Extreme Right</v>
+        <v>Left</v>
       </c>
       <c r="M43" t="str">
         <v>Left</v>
@@ -3635,10 +4055,10 @@
         <v>0</v>
       </c>
       <c r="O43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q43">
         <v>0</v>
@@ -3647,45 +4067,45 @@
         <v>0</v>
       </c>
       <c r="S43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T43">
         <v>0</v>
       </c>
       <c r="U43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V43">
         <v>0</v>
       </c>
       <c r="W43" t="str">
-        <v>RI:L1= DN LL</v>
+        <v/>
       </c>
       <c r="X43" t="str">
-        <v>Book shows one left arm on top of vertical stem</v>
+        <v/>
       </c>
       <c r="Y43">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="Z43">
         <v>1</v>
       </c>
       <c r="AA43" t="str">
-        <v>94/18</v>
+        <v>86/10</v>
       </c>
       <c r="AB43" t="str">
-        <v>Home</v>
+        <v>Advance Starter</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ATG S-12</v>
+        <v>ASO IBS DIST</v>
       </c>
       <c r="B44" t="str">
-        <v>ATG</v>
+        <v/>
       </c>
       <c r="C44" t="str">
-        <v>Atgaon</v>
+        <v/>
       </c>
       <c r="D44" t="str">
         <v>KYN-KSRA</v>
@@ -3697,16 +4117,16 @@
         <v>DN</v>
       </c>
       <c r="G44" t="str">
-        <v>95/24</v>
+        <v>89/2</v>
       </c>
       <c r="H44">
-        <v>95.219</v>
+        <v>88.833</v>
       </c>
       <c r="I44">
-        <v>19.50733</v>
+        <v>19.47014</v>
       </c>
       <c r="J44">
-        <v>73.32688</v>
+        <v>73.30104</v>
       </c>
       <c r="K44" t="str">
         <v>Manual</v>
@@ -3744,28 +4164,34 @@
       <c r="V44">
         <v>0</v>
       </c>
+      <c r="W44" t="str">
+        <v/>
+      </c>
+      <c r="X44" t="str">
+        <v/>
+      </c>
       <c r="Y44">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="Z44">
         <v>1</v>
       </c>
       <c r="AA44" t="str">
-        <v>95/24</v>
+        <v>89/2</v>
       </c>
       <c r="AB44" t="str">
-        <v>Starter</v>
+        <v>IBS Distant</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ATG S-13</v>
+        <v>ASO S-14</v>
       </c>
       <c r="B45" t="str">
-        <v>ATG</v>
+        <v/>
       </c>
       <c r="C45" t="str">
-        <v>Atgaon</v>
+        <v/>
       </c>
       <c r="D45" t="str">
         <v>KYN-KSRA</v>
@@ -3777,16 +4203,16 @@
         <v>DN</v>
       </c>
       <c r="G45" t="str">
-        <v>95/44</v>
+        <v>90/12</v>
       </c>
       <c r="H45">
-        <v>95.62299999999999</v>
+        <v>90.033</v>
       </c>
       <c r="I45">
-        <v>19.51091</v>
+        <v>19.47645</v>
       </c>
       <c r="J45">
-        <v>73.32754</v>
+        <v>73.30968</v>
       </c>
       <c r="K45" t="str">
         <v>Manual</v>
@@ -3824,22 +4250,34 @@
       <c r="V45">
         <v>0</v>
       </c>
+      <c r="W45" t="str">
+        <v/>
+      </c>
+      <c r="X45" t="str">
+        <v/>
+      </c>
       <c r="Y45">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="Z45">
         <v>1</v>
       </c>
       <c r="AA45" t="str">
-        <v>95/44</v>
+        <v>90/12</v>
       </c>
       <c r="AB45" t="str">
-        <v>Advance Starter</v>
+        <v>IBS</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ATG IBS DIST</v>
+        <v>Gate-69 DIST</v>
+      </c>
+      <c r="B46" t="str">
+        <v/>
+      </c>
+      <c r="C46" t="str">
+        <v/>
       </c>
       <c r="D46" t="str">
         <v>KYN-KSRA</v>
@@ -3851,16 +4289,16 @@
         <v>DN</v>
       </c>
       <c r="G46" t="str">
-        <v>96/26</v>
+        <v>91/44</v>
       </c>
       <c r="H46">
-        <v>96.36</v>
+        <v>91.613</v>
       </c>
       <c r="I46">
-        <v>19.51557</v>
+        <v>19.48589</v>
       </c>
       <c r="J46">
-        <v>73.33236</v>
+        <v>73.31983</v>
       </c>
       <c r="K46" t="str">
         <v>Manual</v>
@@ -3869,7 +4307,7 @@
         <v>Left</v>
       </c>
       <c r="M46" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="N46">
         <v>0</v>
@@ -3897,6 +4335,12 @@
       </c>
       <c r="V46">
         <v>0</v>
+      </c>
+      <c r="W46" t="str">
+        <v/>
+      </c>
+      <c r="X46" t="str">
+        <v/>
       </c>
       <c r="Y46">
         <v>450</v>
@@ -3905,15 +4349,21 @@
         <v>1</v>
       </c>
       <c r="AA46" t="str">
-        <v>96/26</v>
+        <v>91/44</v>
       </c>
       <c r="AB46" t="str">
-        <v>IBS Distant</v>
+        <v>Distant</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ATG S-14</v>
+        <v>Gate-69</v>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47" t="str">
+        <v/>
       </c>
       <c r="D47" t="str">
         <v>KYN-KSRA</v>
@@ -3925,34 +4375,34 @@
         <v>DN</v>
       </c>
       <c r="G47" t="str">
-        <v>98/06</v>
+        <v>92/40</v>
       </c>
       <c r="H47">
-        <v>97.94</v>
+        <v>92.60900000000001</v>
       </c>
       <c r="I47">
-        <v>19.5283</v>
+        <v>19.4873</v>
       </c>
       <c r="J47">
-        <v>73.33822</v>
+        <v>73.32914</v>
       </c>
       <c r="K47" t="str">
-        <v>Manual</v>
+        <v>Gate</v>
       </c>
       <c r="L47" t="str">
-        <v>Left</v>
+        <v>Extreme Right</v>
       </c>
       <c r="M47" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="N47">
         <v>0</v>
       </c>
       <c r="O47">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q47">
         <v>0</v>
@@ -3972,28 +4422,34 @@
       <c r="V47">
         <v>0</v>
       </c>
+      <c r="W47" t="str">
+        <v/>
+      </c>
+      <c r="X47" t="str">
+        <v/>
+      </c>
       <c r="Y47">
-        <v>700</v>
+        <v>300</v>
       </c>
       <c r="Z47">
         <v>1</v>
       </c>
       <c r="AA47" t="str">
-        <v>98/06</v>
+        <v>92/40</v>
       </c>
       <c r="AB47" t="str">
-        <v>IBS</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>THS DIST</v>
+        <v>ATG S-3</v>
       </c>
       <c r="B48" t="str">
-        <v>THS</v>
+        <v>ATG</v>
       </c>
       <c r="C48" t="str">
-        <v>Thansit</v>
+        <v>Atgaon</v>
       </c>
       <c r="D48" t="str">
         <v>KYN-KSRA</v>
@@ -4005,22 +4461,22 @@
         <v>DN</v>
       </c>
       <c r="G48" t="str">
-        <v>100/2</v>
+        <v>94/18</v>
       </c>
       <c r="H48">
-        <v>99.88</v>
+        <v>94.089</v>
       </c>
       <c r="I48">
-        <v>19.54288</v>
+        <v>19.4989</v>
       </c>
       <c r="J48">
-        <v>73.34836</v>
+        <v>73.33237</v>
       </c>
       <c r="K48" t="str">
         <v>Manual</v>
       </c>
       <c r="L48" t="str">
-        <v>Left</v>
+        <v>Extreme Right</v>
       </c>
       <c r="M48" t="str">
         <v>Left</v>
@@ -4029,10 +4485,10 @@
         <v>0</v>
       </c>
       <c r="O48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q48">
         <v>0</v>
@@ -4041,39 +4497,45 @@
         <v>0</v>
       </c>
       <c r="S48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T48">
         <v>0</v>
       </c>
       <c r="U48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V48">
         <v>0</v>
       </c>
+      <c r="W48" t="str">
+        <v>RI:L1= DN LL</v>
+      </c>
+      <c r="X48" t="str">
+        <v>Book shows one left arm on top of vertical stem</v>
+      </c>
       <c r="Y48">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="Z48">
         <v>1</v>
       </c>
       <c r="AA48" t="str">
-        <v>100/2</v>
+        <v>94/18</v>
       </c>
       <c r="AB48" t="str">
-        <v>Distant</v>
+        <v>Home</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>THS S-2</v>
+        <v>ATG S-12</v>
       </c>
       <c r="B49" t="str">
-        <v>THS</v>
+        <v>ATG</v>
       </c>
       <c r="C49" t="str">
-        <v>Thansit</v>
+        <v>Atgaon</v>
       </c>
       <c r="D49" t="str">
         <v>KYN-KSRA</v>
@@ -4085,16 +4547,16 @@
         <v>DN</v>
       </c>
       <c r="G49" t="str">
-        <v>101/06</v>
+        <v>95/24</v>
       </c>
       <c r="H49">
-        <v>101.03</v>
+        <v>95.219</v>
       </c>
       <c r="I49">
-        <v>19.55225</v>
+        <v>19.50733</v>
       </c>
       <c r="J49">
-        <v>73.35287</v>
+        <v>73.32688</v>
       </c>
       <c r="K49" t="str">
         <v>Manual</v>
@@ -4103,7 +4565,7 @@
         <v>Left</v>
       </c>
       <c r="M49" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="N49">
         <v>0</v>
@@ -4132,28 +4594,34 @@
       <c r="V49">
         <v>0</v>
       </c>
+      <c r="W49" t="str">
+        <v/>
+      </c>
+      <c r="X49" t="str">
+        <v/>
+      </c>
       <c r="Y49">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="Z49">
         <v>1</v>
       </c>
       <c r="AA49" t="str">
-        <v>101/06</v>
+        <v>95/24</v>
       </c>
       <c r="AB49" t="str">
-        <v>Home</v>
+        <v>Starter</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>THS IBS DIST</v>
+        <v>ATG S-11</v>
       </c>
       <c r="B50" t="str">
-        <v>THS</v>
+        <v>ATG</v>
       </c>
       <c r="C50" t="str">
-        <v>Thansit</v>
+        <v>Atgaon</v>
       </c>
       <c r="D50" t="str">
         <v>KYN-KSRA</v>
@@ -4165,16 +4633,16 @@
         <v>DN</v>
       </c>
       <c r="G50" t="str">
-        <v>102/38</v>
+        <v>DN LOOP STR</v>
       </c>
       <c r="H50">
-        <v>102.68</v>
-      </c>
-      <c r="I50">
-        <v>19.56628</v>
-      </c>
-      <c r="J50">
-        <v>73.35793</v>
+        <v>95.219</v>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
       </c>
       <c r="K50" t="str">
         <v>Manual</v>
@@ -4183,7 +4651,7 @@
         <v>Left</v>
       </c>
       <c r="M50" t="str">
-        <v>Right</v>
+        <v/>
       </c>
       <c r="N50">
         <v>0</v>
@@ -4212,28 +4680,34 @@
       <c r="V50">
         <v>0</v>
       </c>
-      <c r="Y50">
-        <v>600</v>
+      <c r="W50" t="str">
+        <v/>
+      </c>
+      <c r="X50" t="str">
+        <v/>
+      </c>
+      <c r="Y50" t="str">
+        <v/>
       </c>
       <c r="Z50">
         <v>1</v>
       </c>
       <c r="AA50" t="str">
-        <v>102/38</v>
+        <v>95/24</v>
       </c>
       <c r="AB50" t="str">
-        <v>IBS Distant</v>
+        <v>Starter (Loop)</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>THS S-5</v>
+        <v>ATG S-13</v>
       </c>
       <c r="B51" t="str">
-        <v>THS</v>
+        <v>ATG</v>
       </c>
       <c r="C51" t="str">
-        <v>Thansit</v>
+        <v>Atgaon</v>
       </c>
       <c r="D51" t="str">
         <v>KYN-KSRA</v>
@@ -4245,16 +4719,16 @@
         <v>DN</v>
       </c>
       <c r="G51" t="str">
-        <v>103/38</v>
+        <v>95/44</v>
       </c>
       <c r="H51">
-        <v>103.673</v>
+        <v>95.62299999999999</v>
       </c>
       <c r="I51">
-        <v>19.56628</v>
+        <v>19.51091</v>
       </c>
       <c r="J51">
-        <v>73.35793</v>
+        <v>73.32754</v>
       </c>
       <c r="K51" t="str">
         <v>Manual</v>
@@ -4292,28 +4766,34 @@
       <c r="V51">
         <v>0</v>
       </c>
+      <c r="W51" t="str">
+        <v/>
+      </c>
+      <c r="X51" t="str">
+        <v/>
+      </c>
       <c r="Y51">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="Z51">
         <v>1</v>
       </c>
       <c r="AA51" t="str">
-        <v>103/38</v>
+        <v>95/44</v>
       </c>
       <c r="AB51" t="str">
-        <v>IBS</v>
+        <v>Advance Starter</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>KE DIST</v>
+        <v>ATG IBS DIST</v>
       </c>
       <c r="B52" t="str">
-        <v>KE</v>
+        <v/>
       </c>
       <c r="C52" t="str">
-        <v>Khardi</v>
+        <v/>
       </c>
       <c r="D52" t="str">
         <v>KYN-KSRA</v>
@@ -4325,16 +4805,16 @@
         <v>DN</v>
       </c>
       <c r="G52" t="str">
-        <v>105/08</v>
+        <v>96/26</v>
       </c>
       <c r="H52">
-        <v>105.003</v>
+        <v>96.36</v>
       </c>
       <c r="I52">
-        <v>19.57563</v>
+        <v>19.51557</v>
       </c>
       <c r="J52">
-        <v>73.37633</v>
+        <v>73.33236</v>
       </c>
       <c r="K52" t="str">
         <v>Manual</v>
@@ -4343,7 +4823,7 @@
         <v>Left</v>
       </c>
       <c r="M52" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="N52">
         <v>0</v>
@@ -4372,28 +4852,34 @@
       <c r="V52">
         <v>0</v>
       </c>
+      <c r="W52" t="str">
+        <v/>
+      </c>
+      <c r="X52" t="str">
+        <v/>
+      </c>
       <c r="Y52">
-        <v>415</v>
+        <v>450</v>
       </c>
       <c r="Z52">
         <v>1</v>
       </c>
       <c r="AA52" t="str">
-        <v>105/08</v>
+        <v>96/26</v>
       </c>
       <c r="AB52" t="str">
-        <v>Distant</v>
+        <v>IBS Distant</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>KE S-3</v>
+        <v>ATG S-14</v>
       </c>
       <c r="B53" t="str">
-        <v>KE</v>
+        <v/>
       </c>
       <c r="C53" t="str">
-        <v>Khardi</v>
+        <v/>
       </c>
       <c r="D53" t="str">
         <v>KYN-KSRA</v>
@@ -4405,16 +4891,16 @@
         <v>DN</v>
       </c>
       <c r="G53" t="str">
-        <v>106/08</v>
+        <v>98/06</v>
       </c>
       <c r="H53">
-        <v>106.083</v>
+        <v>97.94</v>
       </c>
       <c r="I53">
-        <v>19.57874</v>
+        <v>19.5283</v>
       </c>
       <c r="J53">
-        <v>73.38608</v>
+        <v>73.33822</v>
       </c>
       <c r="K53" t="str">
         <v>Manual</v>
@@ -4441,45 +4927,45 @@
         <v>0</v>
       </c>
       <c r="S53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T53">
         <v>0</v>
       </c>
       <c r="U53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V53">
         <v>0</v>
       </c>
       <c r="W53" t="str">
-        <v>RI:L1= DN LL</v>
+        <v/>
       </c>
       <c r="X53" t="str">
-        <v>Book shows one left arm on top of vertical stem</v>
+        <v/>
       </c>
       <c r="Y53">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="Z53">
         <v>1</v>
       </c>
       <c r="AA53" t="str">
-        <v>106/08</v>
+        <v>98/06</v>
       </c>
       <c r="AB53" t="str">
-        <v>Home</v>
+        <v>IBS</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>KE S-12</v>
+        <v>THS DIST</v>
       </c>
       <c r="B54" t="str">
-        <v>KE</v>
+        <v>THS</v>
       </c>
       <c r="C54" t="str">
-        <v>Khardi</v>
+        <v>Thansit</v>
       </c>
       <c r="D54" t="str">
         <v>KYN-KSRA</v>
@@ -4491,22 +4977,22 @@
         <v>DN</v>
       </c>
       <c r="G54" t="str">
-        <v>107/24</v>
+        <v>100/2</v>
       </c>
       <c r="H54">
-        <v>107.32300000000001</v>
+        <v>99.88</v>
       </c>
       <c r="I54">
-        <v>19.58287</v>
+        <v>19.54288</v>
       </c>
       <c r="J54">
-        <v>73.39642</v>
+        <v>73.34836</v>
       </c>
       <c r="K54" t="str">
         <v>Manual</v>
       </c>
       <c r="L54" t="str">
-        <v>Extreme Right</v>
+        <v>Left</v>
       </c>
       <c r="M54" t="str">
         <v>Left</v>
@@ -4515,10 +5001,10 @@
         <v>0</v>
       </c>
       <c r="O54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q54">
         <v>0</v>
@@ -4538,28 +5024,34 @@
       <c r="V54">
         <v>0</v>
       </c>
+      <c r="W54" t="str">
+        <v/>
+      </c>
+      <c r="X54" t="str">
+        <v/>
+      </c>
       <c r="Y54">
-        <v>245</v>
+        <v>500</v>
       </c>
       <c r="Z54">
         <v>1</v>
       </c>
       <c r="AA54" t="str">
-        <v>107/24</v>
+        <v>100/2</v>
       </c>
       <c r="AB54" t="str">
-        <v>Starter</v>
+        <v>Distant</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>KE S-13</v>
+        <v>THS S-2</v>
       </c>
       <c r="B55" t="str">
-        <v>KE</v>
+        <v>THS</v>
       </c>
       <c r="C55" t="str">
-        <v>Khardi</v>
+        <v>Thansit</v>
       </c>
       <c r="D55" t="str">
         <v>KYN-KSRA</v>
@@ -4571,16 +5063,16 @@
         <v>DN</v>
       </c>
       <c r="G55" t="str">
-        <v>107/44</v>
+        <v>101/06</v>
       </c>
       <c r="H55">
-        <v>107.78999999999999</v>
+        <v>101.03</v>
       </c>
       <c r="I55">
-        <v>19.58661</v>
+        <v>19.55225</v>
       </c>
       <c r="J55">
-        <v>73.39847</v>
+        <v>73.35287</v>
       </c>
       <c r="K55" t="str">
         <v>Manual</v>
@@ -4618,22 +5110,34 @@
       <c r="V55">
         <v>0</v>
       </c>
+      <c r="W55" t="str">
+        <v/>
+      </c>
+      <c r="X55" t="str">
+        <v/>
+      </c>
       <c r="Y55">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="Z55">
         <v>1</v>
       </c>
       <c r="AA55" t="str">
-        <v>107/44</v>
+        <v>101/06</v>
       </c>
       <c r="AB55" t="str">
-        <v>Advance Starter</v>
+        <v>Home</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>KE IBS DIST</v>
+        <v>THS IBS DIST</v>
+      </c>
+      <c r="B56" t="str">
+        <v>THS</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Thansit</v>
       </c>
       <c r="D56" t="str">
         <v>KYN-KSRA</v>
@@ -4645,16 +5149,16 @@
         <v>DN</v>
       </c>
       <c r="G56" t="str">
-        <v>109/06</v>
+        <v>102/38</v>
       </c>
       <c r="H56">
-        <v>108.95</v>
+        <v>102.68</v>
       </c>
       <c r="I56">
-        <v>19.59682</v>
+        <v>19.56628</v>
       </c>
       <c r="J56">
-        <v>73.39948</v>
+        <v>73.35793</v>
       </c>
       <c r="K56" t="str">
         <v>Manual</v>
@@ -4663,7 +5167,7 @@
         <v>Left</v>
       </c>
       <c r="M56" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="N56">
         <v>0</v>
@@ -4692,14 +5196,20 @@
       <c r="V56">
         <v>0</v>
       </c>
+      <c r="W56" t="str">
+        <v/>
+      </c>
+      <c r="X56" t="str">
+        <v/>
+      </c>
       <c r="Y56">
-        <v>410</v>
+        <v>600</v>
       </c>
       <c r="Z56">
         <v>1</v>
       </c>
       <c r="AA56" t="str">
-        <v>109/06</v>
+        <v>102/38</v>
       </c>
       <c r="AB56" t="str">
         <v>IBS Distant</v>
@@ -4707,13 +5217,13 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>KE S-14</v>
+        <v>THS S-5</v>
       </c>
       <c r="B57" t="str">
-        <v>KE</v>
+        <v>THS</v>
       </c>
       <c r="C57" t="str">
-        <v>Khardi</v>
+        <v>Thansit</v>
       </c>
       <c r="D57" t="str">
         <v>KYN-KSRA</v>
@@ -4725,16 +5235,16 @@
         <v>DN</v>
       </c>
       <c r="G57" t="str">
-        <v>110/06</v>
+        <v>103/38</v>
       </c>
       <c r="H57">
-        <v>109.96000000000001</v>
+        <v>103.673</v>
       </c>
       <c r="I57">
-        <v>19.60556</v>
+        <v>19.56628</v>
       </c>
       <c r="J57">
-        <v>73.40126</v>
+        <v>73.35793</v>
       </c>
       <c r="K57" t="str">
         <v>Manual</v>
@@ -4772,6 +5282,12 @@
       <c r="V57">
         <v>0</v>
       </c>
+      <c r="W57" t="str">
+        <v/>
+      </c>
+      <c r="X57" t="str">
+        <v/>
+      </c>
       <c r="Y57">
         <v>400</v>
       </c>
@@ -4779,7 +5295,7 @@
         <v>1</v>
       </c>
       <c r="AA57" t="str">
-        <v>110/06</v>
+        <v>103/38</v>
       </c>
       <c r="AB57" t="str">
         <v>IBS</v>
@@ -4787,13 +5303,13 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>OMB DIST</v>
+        <v>KE DIST</v>
       </c>
       <c r="B58" t="str">
-        <v>OMB</v>
+        <v>KE</v>
       </c>
       <c r="C58" t="str">
-        <v>Umbermali</v>
+        <v>Khardi</v>
       </c>
       <c r="D58" t="str">
         <v>KYN-KSRA</v>
@@ -4805,16 +5321,16 @@
         <v>DN</v>
       </c>
       <c r="G58" t="str">
-        <v>112/14</v>
+        <v>105/08</v>
       </c>
       <c r="H58">
-        <v>112.15</v>
+        <v>105.003</v>
       </c>
       <c r="I58">
-        <v>19.61798</v>
+        <v>19.57563</v>
       </c>
       <c r="J58">
-        <v>73.41725</v>
+        <v>73.37633</v>
       </c>
       <c r="K58" t="str">
         <v>Manual</v>
@@ -4823,7 +5339,7 @@
         <v>Left</v>
       </c>
       <c r="M58" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="N58">
         <v>0</v>
@@ -4852,14 +5368,20 @@
       <c r="V58">
         <v>0</v>
       </c>
+      <c r="W58" t="str">
+        <v/>
+      </c>
+      <c r="X58" t="str">
+        <v/>
+      </c>
       <c r="Y58">
-        <v>500</v>
+        <v>415</v>
       </c>
       <c r="Z58">
         <v>1</v>
       </c>
       <c r="AA58" t="str">
-        <v>112/14</v>
+        <v>105/08</v>
       </c>
       <c r="AB58" t="str">
         <v>Distant</v>
@@ -4867,13 +5389,13 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>OMB S-2</v>
+        <v>KE S-3</v>
       </c>
       <c r="B59" t="str">
-        <v>OMB</v>
+        <v>KE</v>
       </c>
       <c r="C59" t="str">
-        <v>Umbermali</v>
+        <v>Khardi</v>
       </c>
       <c r="D59" t="str">
         <v>KYN-KSRA</v>
@@ -4885,16 +5407,16 @@
         <v>DN</v>
       </c>
       <c r="G59" t="str">
-        <v>113/26</v>
+        <v>106/08</v>
       </c>
       <c r="H59">
-        <v>113.23</v>
+        <v>106.083</v>
       </c>
       <c r="I59">
-        <v>19.62628</v>
+        <v>19.57874</v>
       </c>
       <c r="J59">
-        <v>73.42169</v>
+        <v>73.38608</v>
       </c>
       <c r="K59" t="str">
         <v>Manual</v>
@@ -4903,7 +5425,7 @@
         <v>Left</v>
       </c>
       <c r="M59" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="N59">
         <v>0</v>
@@ -4921,25 +5443,31 @@
         <v>0</v>
       </c>
       <c r="S59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T59">
         <v>0</v>
       </c>
       <c r="U59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V59">
         <v>0</v>
       </c>
+      <c r="W59" t="str">
+        <v>RI:L1= DN LL</v>
+      </c>
+      <c r="X59" t="str">
+        <v>Book shows one left arm on top of vertical stem</v>
+      </c>
       <c r="Y59">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="Z59">
         <v>1</v>
       </c>
       <c r="AA59" t="str">
-        <v>113/26</v>
+        <v>106/08</v>
       </c>
       <c r="AB59" t="str">
         <v>Home</v>
@@ -4947,7 +5475,13 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>OMB IBS DIST</v>
+        <v>KE S-12</v>
+      </c>
+      <c r="B60" t="str">
+        <v>KE</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Khardi</v>
       </c>
       <c r="D60" t="str">
         <v>KYN-KSRA</v>
@@ -4959,34 +5493,34 @@
         <v>DN</v>
       </c>
       <c r="G60" t="str">
-        <v>115/50</v>
+        <v>107/24</v>
       </c>
       <c r="H60">
-        <v>115.78</v>
+        <v>107.32300000000001</v>
       </c>
       <c r="I60">
-        <v>19.63105</v>
+        <v>19.58287</v>
       </c>
       <c r="J60">
-        <v>73.44172</v>
+        <v>73.39642</v>
       </c>
       <c r="K60" t="str">
         <v>Manual</v>
       </c>
       <c r="L60" t="str">
-        <v>Left</v>
+        <v>Extreme Right</v>
       </c>
       <c r="M60" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="N60">
         <v>0</v>
       </c>
       <c r="O60">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q60">
         <v>0</v>
@@ -5006,22 +5540,34 @@
       <c r="V60">
         <v>0</v>
       </c>
+      <c r="W60" t="str">
+        <v/>
+      </c>
+      <c r="X60" t="str">
+        <v/>
+      </c>
       <c r="Y60">
-        <v>450</v>
+        <v>245</v>
       </c>
       <c r="Z60">
         <v>1</v>
       </c>
       <c r="AA60" t="str">
-        <v>115/50</v>
+        <v>107/24</v>
       </c>
       <c r="AB60" t="str">
-        <v>IBS Distant</v>
+        <v>Starter</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>OMB S-5</v>
+        <v>KE S-11</v>
+      </c>
+      <c r="B61" t="str">
+        <v>KE</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Khardi</v>
       </c>
       <c r="D61" t="str">
         <v>KYN-KSRA</v>
@@ -5033,16 +5579,16 @@
         <v>DN</v>
       </c>
       <c r="G61" t="str">
-        <v>117/04</v>
-      </c>
-      <c r="H61">
-        <v>116.89</v>
-      </c>
-      <c r="I61">
-        <v>19.6292</v>
-      </c>
-      <c r="J61">
-        <v>73.4512</v>
+        <v>DN LOOP STR</v>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+      <c r="I61" t="str">
+        <v/>
+      </c>
+      <c r="J61" t="str">
+        <v/>
       </c>
       <c r="K61" t="str">
         <v>Manual</v>
@@ -5051,7 +5597,7 @@
         <v>Left</v>
       </c>
       <c r="M61" t="str">
-        <v>Left</v>
+        <v/>
       </c>
       <c r="N61">
         <v>0</v>
@@ -5080,28 +5626,34 @@
       <c r="V61">
         <v>0</v>
       </c>
-      <c r="Y61">
-        <v>300</v>
+      <c r="W61" t="str">
+        <v/>
+      </c>
+      <c r="X61" t="str">
+        <v/>
+      </c>
+      <c r="Y61" t="str">
+        <v/>
       </c>
       <c r="Z61">
         <v>1</v>
       </c>
       <c r="AA61" t="str">
-        <v>117/04</v>
+        <v>107/1008</v>
       </c>
       <c r="AB61" t="str">
-        <v>IBS</v>
+        <v>Starter (Loop)</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>KSRA DIST</v>
+        <v>KE S-13</v>
       </c>
       <c r="B62" t="str">
-        <v>KSRA</v>
+        <v>KE</v>
       </c>
       <c r="C62" t="str">
-        <v>Kasara</v>
+        <v>Khardi</v>
       </c>
       <c r="D62" t="str">
         <v>KYN-KSRA</v>
@@ -5113,16 +5665,16 @@
         <v>DN</v>
       </c>
       <c r="G62" t="str">
-        <v>118/16</v>
+        <v>107/44</v>
       </c>
       <c r="H62">
-        <v>118.1</v>
+        <v>107.78999999999999</v>
       </c>
       <c r="I62">
-        <v>19.63443</v>
+        <v>19.58661</v>
       </c>
       <c r="J62">
-        <v>73.46043</v>
+        <v>73.39847</v>
       </c>
       <c r="K62" t="str">
         <v>Manual</v>
@@ -5131,7 +5683,7 @@
         <v>Left</v>
       </c>
       <c r="M62" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="N62">
         <v>0</v>
@@ -5160,28 +5712,34 @@
       <c r="V62">
         <v>0</v>
       </c>
+      <c r="W62" t="str">
+        <v/>
+      </c>
+      <c r="X62" t="str">
+        <v/>
+      </c>
       <c r="Y62">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="Z62">
         <v>1</v>
       </c>
       <c r="AA62" t="str">
-        <v>118/16</v>
+        <v>107/44</v>
       </c>
       <c r="AB62" t="str">
-        <v>Distant</v>
+        <v>Advance Starter</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>KSRA S-2</v>
+        <v>KE IBS DIST</v>
       </c>
       <c r="B63" t="str">
-        <v>KSRA</v>
+        <v/>
       </c>
       <c r="C63" t="str">
-        <v>Kasara</v>
+        <v/>
       </c>
       <c r="D63" t="str">
         <v>KYN-KSRA</v>
@@ -5193,22 +5751,22 @@
         <v>DN</v>
       </c>
       <c r="G63" t="str">
-        <v>119/16</v>
+        <v>109/06</v>
       </c>
       <c r="H63">
-        <v>119.096</v>
+        <v>108.95</v>
       </c>
       <c r="I63">
-        <v>19.63764</v>
+        <v>19.59682</v>
       </c>
       <c r="J63">
-        <v>73.46852</v>
+        <v>73.39948</v>
       </c>
       <c r="K63" t="str">
         <v>Manual</v>
       </c>
       <c r="L63" t="str">
-        <v>Extreme Right</v>
+        <v>Left</v>
       </c>
       <c r="M63" t="str">
         <v>Left</v>
@@ -5217,10 +5775,10 @@
         <v>0</v>
       </c>
       <c r="O63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q63">
         <v>0</v>
@@ -5229,45 +5787,45 @@
         <v>0</v>
       </c>
       <c r="S63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T63">
         <v>0</v>
       </c>
       <c r="U63">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V63">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W63" t="str">
-        <v>RI:L1= RD-3; L2=RD-2; L3=RD-1; R1=; R2=; R3=</v>
+        <v/>
       </c>
       <c r="X63" t="str">
-        <v>Book shows three left and three right arms on top of vertical stem</v>
+        <v/>
       </c>
       <c r="Y63">
-        <v>250</v>
+        <v>410</v>
       </c>
       <c r="Z63">
         <v>1</v>
       </c>
       <c r="AA63" t="str">
-        <v>119/16</v>
+        <v>109/06</v>
       </c>
       <c r="AB63" t="str">
-        <v>Home</v>
+        <v>IBS Distant</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>KSRA S-46</v>
+        <v>KE S-14</v>
       </c>
       <c r="B64" t="str">
-        <v>KSRA</v>
+        <v>KE</v>
       </c>
       <c r="C64" t="str">
-        <v>Kasara</v>
+        <v>Khardi</v>
       </c>
       <c r="D64" t="str">
         <v>KYN-KSRA</v>
@@ -5279,75 +5837,677 @@
         <v>DN</v>
       </c>
       <c r="G64" t="str">
-        <v>PF-1 STR</v>
+        <v>110/06</v>
       </c>
       <c r="H64">
-        <v>120.666</v>
+        <v>109.96000000000001</v>
       </c>
       <c r="I64">
-        <v>19.6508</v>
+        <v>19.60556</v>
       </c>
       <c r="J64">
-        <v>73.47375</v>
+        <v>73.40126</v>
       </c>
       <c r="K64" t="str">
         <v>Manual</v>
       </c>
       <c r="L64" t="str">
+        <v>Left</v>
+      </c>
+      <c r="M64" t="str">
         <v>Right</v>
       </c>
-      <c r="M64" t="str">
+      <c r="N64">
+        <v>0</v>
+      </c>
+      <c r="O64">
+        <v>0</v>
+      </c>
+      <c r="P64">
+        <v>1</v>
+      </c>
+      <c r="Q64">
+        <v>0</v>
+      </c>
+      <c r="R64">
+        <v>0</v>
+      </c>
+      <c r="S64">
+        <v>0</v>
+      </c>
+      <c r="T64">
+        <v>0</v>
+      </c>
+      <c r="U64">
+        <v>0</v>
+      </c>
+      <c r="V64">
+        <v>0</v>
+      </c>
+      <c r="W64" t="str">
+        <v/>
+      </c>
+      <c r="X64" t="str">
+        <v/>
+      </c>
+      <c r="Y64">
+        <v>400</v>
+      </c>
+      <c r="Z64">
+        <v>1</v>
+      </c>
+      <c r="AA64" t="str">
+        <v>110/06</v>
+      </c>
+      <c r="AB64" t="str">
+        <v>IBS</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>OMB DIST</v>
+      </c>
+      <c r="B65" t="str">
+        <v>OMB</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Umbermali</v>
+      </c>
+      <c r="D65" t="str">
+        <v>KYN-KSRA</v>
+      </c>
+      <c r="E65" t="str">
+        <v>DN NE</v>
+      </c>
+      <c r="F65" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G65" t="str">
+        <v>112/14</v>
+      </c>
+      <c r="H65">
+        <v>112.15</v>
+      </c>
+      <c r="I65">
+        <v>19.61798</v>
+      </c>
+      <c r="J65">
+        <v>73.41725</v>
+      </c>
+      <c r="K65" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="L65" t="str">
+        <v>Left</v>
+      </c>
+      <c r="M65" t="str">
+        <v>Right</v>
+      </c>
+      <c r="N65">
+        <v>0</v>
+      </c>
+      <c r="O65">
+        <v>0</v>
+      </c>
+      <c r="P65">
+        <v>1</v>
+      </c>
+      <c r="Q65">
+        <v>0</v>
+      </c>
+      <c r="R65">
+        <v>0</v>
+      </c>
+      <c r="S65">
+        <v>0</v>
+      </c>
+      <c r="T65">
+        <v>0</v>
+      </c>
+      <c r="U65">
+        <v>0</v>
+      </c>
+      <c r="V65">
+        <v>0</v>
+      </c>
+      <c r="W65" t="str">
+        <v/>
+      </c>
+      <c r="X65" t="str">
+        <v/>
+      </c>
+      <c r="Y65">
+        <v>500</v>
+      </c>
+      <c r="Z65">
+        <v>1</v>
+      </c>
+      <c r="AA65" t="str">
+        <v>112/14</v>
+      </c>
+      <c r="AB65" t="str">
+        <v>Distant</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>OMB S-2</v>
+      </c>
+      <c r="B66" t="str">
+        <v>OMB</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Umbermali</v>
+      </c>
+      <c r="D66" t="str">
+        <v>KYN-KSRA</v>
+      </c>
+      <c r="E66" t="str">
+        <v>DN NE</v>
+      </c>
+      <c r="F66" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G66" t="str">
+        <v>113/26</v>
+      </c>
+      <c r="H66">
+        <v>113.23</v>
+      </c>
+      <c r="I66">
+        <v>19.62628</v>
+      </c>
+      <c r="J66">
+        <v>73.42169</v>
+      </c>
+      <c r="K66" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="L66" t="str">
+        <v>Left</v>
+      </c>
+      <c r="M66" t="str">
+        <v>Left</v>
+      </c>
+      <c r="N66">
+        <v>0</v>
+      </c>
+      <c r="O66">
+        <v>0</v>
+      </c>
+      <c r="P66">
+        <v>1</v>
+      </c>
+      <c r="Q66">
+        <v>0</v>
+      </c>
+      <c r="R66">
+        <v>0</v>
+      </c>
+      <c r="S66">
+        <v>0</v>
+      </c>
+      <c r="T66">
+        <v>0</v>
+      </c>
+      <c r="U66">
+        <v>0</v>
+      </c>
+      <c r="V66">
+        <v>0</v>
+      </c>
+      <c r="W66" t="str">
+        <v/>
+      </c>
+      <c r="X66" t="str">
+        <v/>
+      </c>
+      <c r="Y66">
+        <v>350</v>
+      </c>
+      <c r="Z66">
+        <v>1</v>
+      </c>
+      <c r="AA66" t="str">
+        <v>113/26</v>
+      </c>
+      <c r="AB66" t="str">
+        <v>Home</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>OMB IBS DIST</v>
+      </c>
+      <c r="B67" t="str">
+        <v/>
+      </c>
+      <c r="C67" t="str">
+        <v/>
+      </c>
+      <c r="D67" t="str">
+        <v>KYN-KSRA</v>
+      </c>
+      <c r="E67" t="str">
+        <v>DN NE</v>
+      </c>
+      <c r="F67" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G67" t="str">
+        <v>115/50</v>
+      </c>
+      <c r="H67">
+        <v>115.78</v>
+      </c>
+      <c r="I67">
+        <v>19.63105</v>
+      </c>
+      <c r="J67">
+        <v>73.44172</v>
+      </c>
+      <c r="K67" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="L67" t="str">
+        <v>Left</v>
+      </c>
+      <c r="M67" t="str">
+        <v>Right</v>
+      </c>
+      <c r="N67">
+        <v>0</v>
+      </c>
+      <c r="O67">
+        <v>0</v>
+      </c>
+      <c r="P67">
+        <v>1</v>
+      </c>
+      <c r="Q67">
+        <v>0</v>
+      </c>
+      <c r="R67">
+        <v>0</v>
+      </c>
+      <c r="S67">
+        <v>0</v>
+      </c>
+      <c r="T67">
+        <v>0</v>
+      </c>
+      <c r="U67">
+        <v>0</v>
+      </c>
+      <c r="V67">
+        <v>0</v>
+      </c>
+      <c r="W67" t="str">
+        <v/>
+      </c>
+      <c r="X67" t="str">
+        <v/>
+      </c>
+      <c r="Y67">
+        <v>450</v>
+      </c>
+      <c r="Z67">
+        <v>1</v>
+      </c>
+      <c r="AA67" t="str">
+        <v>115/50</v>
+      </c>
+      <c r="AB67" t="str">
+        <v>IBS Distant</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>OMB S-5</v>
+      </c>
+      <c r="B68" t="str">
+        <v/>
+      </c>
+      <c r="C68" t="str">
+        <v/>
+      </c>
+      <c r="D68" t="str">
+        <v>KYN-KSRA</v>
+      </c>
+      <c r="E68" t="str">
+        <v>DN NE</v>
+      </c>
+      <c r="F68" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G68" t="str">
+        <v>117/04</v>
+      </c>
+      <c r="H68">
+        <v>116.89</v>
+      </c>
+      <c r="I68">
+        <v>19.6292</v>
+      </c>
+      <c r="J68">
+        <v>73.4512</v>
+      </c>
+      <c r="K68" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="L68" t="str">
+        <v>Left</v>
+      </c>
+      <c r="M68" t="str">
+        <v>Left</v>
+      </c>
+      <c r="N68">
+        <v>0</v>
+      </c>
+      <c r="O68">
+        <v>0</v>
+      </c>
+      <c r="P68">
+        <v>1</v>
+      </c>
+      <c r="Q68">
+        <v>0</v>
+      </c>
+      <c r="R68">
+        <v>0</v>
+      </c>
+      <c r="S68">
+        <v>0</v>
+      </c>
+      <c r="T68">
+        <v>0</v>
+      </c>
+      <c r="U68">
+        <v>0</v>
+      </c>
+      <c r="V68">
+        <v>0</v>
+      </c>
+      <c r="W68" t="str">
+        <v/>
+      </c>
+      <c r="X68" t="str">
+        <v/>
+      </c>
+      <c r="Y68">
+        <v>300</v>
+      </c>
+      <c r="Z68">
+        <v>1</v>
+      </c>
+      <c r="AA68" t="str">
+        <v>117/04</v>
+      </c>
+      <c r="AB68" t="str">
+        <v>IBS</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>KSRA DIST</v>
+      </c>
+      <c r="B69" t="str">
+        <v>KSRA</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Kasara</v>
+      </c>
+      <c r="D69" t="str">
+        <v>KYN-KSRA</v>
+      </c>
+      <c r="E69" t="str">
+        <v>DN NE</v>
+      </c>
+      <c r="F69" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G69" t="str">
+        <v>118/16</v>
+      </c>
+      <c r="H69">
+        <v>118.1</v>
+      </c>
+      <c r="I69">
+        <v>19.63443</v>
+      </c>
+      <c r="J69">
+        <v>73.46043</v>
+      </c>
+      <c r="K69" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="L69" t="str">
+        <v>Left</v>
+      </c>
+      <c r="M69" t="str">
+        <v>Right</v>
+      </c>
+      <c r="N69">
+        <v>0</v>
+      </c>
+      <c r="O69">
+        <v>0</v>
+      </c>
+      <c r="P69">
+        <v>1</v>
+      </c>
+      <c r="Q69">
+        <v>0</v>
+      </c>
+      <c r="R69">
+        <v>0</v>
+      </c>
+      <c r="S69">
+        <v>0</v>
+      </c>
+      <c r="T69">
+        <v>0</v>
+      </c>
+      <c r="U69">
+        <v>0</v>
+      </c>
+      <c r="V69">
+        <v>0</v>
+      </c>
+      <c r="W69" t="str">
+        <v/>
+      </c>
+      <c r="X69" t="str">
+        <v/>
+      </c>
+      <c r="Y69">
+        <v>450</v>
+      </c>
+      <c r="Z69">
+        <v>1</v>
+      </c>
+      <c r="AA69" t="str">
+        <v>118/16</v>
+      </c>
+      <c r="AB69" t="str">
+        <v>Distant</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>KSRA S-2</v>
+      </c>
+      <c r="B70" t="str">
+        <v>KSRA</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Kasara</v>
+      </c>
+      <c r="D70" t="str">
+        <v>KYN-KSRA</v>
+      </c>
+      <c r="E70" t="str">
+        <v>DN NE</v>
+      </c>
+      <c r="F70" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G70" t="str">
+        <v>119/16</v>
+      </c>
+      <c r="H70">
+        <v>119.096</v>
+      </c>
+      <c r="I70">
+        <v>19.63764</v>
+      </c>
+      <c r="J70">
+        <v>73.46852</v>
+      </c>
+      <c r="K70" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="L70" t="str">
+        <v>Extreme Right</v>
+      </c>
+      <c r="M70" t="str">
+        <v>Left</v>
+      </c>
+      <c r="N70">
+        <v>0</v>
+      </c>
+      <c r="O70">
+        <v>1</v>
+      </c>
+      <c r="P70">
+        <v>0</v>
+      </c>
+      <c r="Q70">
+        <v>0</v>
+      </c>
+      <c r="R70">
+        <v>0</v>
+      </c>
+      <c r="S70">
+        <v>1</v>
+      </c>
+      <c r="T70">
+        <v>0</v>
+      </c>
+      <c r="U70">
+        <v>3</v>
+      </c>
+      <c r="V70">
+        <v>3</v>
+      </c>
+      <c r="W70" t="str">
+        <v>RI:L1= RD-3; L2=RD-2; L3=RD-1; R1=; R2=; R3=</v>
+      </c>
+      <c r="X70" t="str">
+        <v>Book shows three left and three right arms on top of vertical stem</v>
+      </c>
+      <c r="Y70">
+        <v>250</v>
+      </c>
+      <c r="Z70">
+        <v>1</v>
+      </c>
+      <c r="AA70" t="str">
+        <v>119/16</v>
+      </c>
+      <c r="AB70" t="str">
+        <v>Home</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>KSRA S-46</v>
+      </c>
+      <c r="B71" t="str">
+        <v>KSRA</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Kasara</v>
+      </c>
+      <c r="D71" t="str">
+        <v>KYN-KSRA</v>
+      </c>
+      <c r="E71" t="str">
+        <v>DN NE</v>
+      </c>
+      <c r="F71" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G71" t="str">
+        <v>PF-1 STR</v>
+      </c>
+      <c r="H71">
+        <v>120.666</v>
+      </c>
+      <c r="I71">
+        <v>19.6508</v>
+      </c>
+      <c r="J71">
+        <v>73.47375</v>
+      </c>
+      <c r="K71" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="L71" t="str">
+        <v>Right</v>
+      </c>
+      <c r="M71" t="str">
         <v>Unknown</v>
       </c>
-      <c r="N64">
-        <v>1</v>
-      </c>
-      <c r="O64">
-        <v>0</v>
-      </c>
-      <c r="P64">
-        <v>0</v>
-      </c>
-      <c r="Q64">
-        <v>0</v>
-      </c>
-      <c r="R64">
-        <v>0</v>
-      </c>
-      <c r="S64">
-        <v>1</v>
-      </c>
-      <c r="T64">
-        <v>1</v>
-      </c>
-      <c r="U64">
-        <v>0</v>
-      </c>
-      <c r="V64">
-        <v>1</v>
-      </c>
-      <c r="W64" t="str">
+      <c r="N71">
+        <v>1</v>
+      </c>
+      <c r="O71">
+        <v>0</v>
+      </c>
+      <c r="P71">
+        <v>0</v>
+      </c>
+      <c r="Q71">
+        <v>0</v>
+      </c>
+      <c r="R71">
+        <v>0</v>
+      </c>
+      <c r="S71">
+        <v>1</v>
+      </c>
+      <c r="T71">
+        <v>1</v>
+      </c>
+      <c r="U71">
+        <v>0</v>
+      </c>
+      <c r="V71">
+        <v>1</v>
+      </c>
+      <c r="W71" t="str">
         <v>RI:R1= DN MID</v>
       </c>
-      <c r="X64" t="str">
+      <c r="X71" t="str">
         <v>Book shows one right arm on top of vertical stem</v>
       </c>
-      <c r="Y64">
+      <c r="Y71">
         <v>300</v>
       </c>
-      <c r="Z64">
-        <v>1</v>
-      </c>
-      <c r="AA64" t="str">
+      <c r="Z71">
+        <v>1</v>
+      </c>
+      <c r="AA71" t="str">
         <v>120/43</v>
       </c>
-      <c r="AB64" t="str">
+      <c r="AB71" t="str">
         <v>Starter</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB71"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>